<commit_message>
docs: validate INF KPIs, add COL KPIs and document CPI pipelines, Job and Power BI
</commit_message>
<xml_diff>
--- a/docs/03_Business_Questions_KPI_Catalog.xlsx
+++ b/docs/03_Business_Questions_KPI_Catalog.xlsx
@@ -691,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -891,7 +891,7 @@
       </c>
       <c r="K5" s="30" t="inlineStr">
         <is>
-          <t>BCRD (to validate)</t>
+          <t>BCRD — IPC base Oct 2019–Sep 2020 workbooks (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L5" s="30" t="inlineStr">
@@ -911,10 +911,14 @@
       </c>
       <c r="O5" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P5" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P5" s="30" t="inlineStr">
+        <is>
+          <t>Base Oct 2019 - Sep 2020 = 100. Series: headline 1984+, groups 1999+, core 2000+, regions 2011+. gold.inflation_metrics.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="30" t="inlineStr">
@@ -969,7 +973,7 @@
       </c>
       <c r="K6" s="30" t="inlineStr">
         <is>
-          <t>BCRD (to validate)</t>
+          <t>BCRD — IPC base Oct 2019–Sep 2020 workbooks (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L6" s="30" t="inlineStr">
@@ -989,10 +993,14 @@
       </c>
       <c r="O6" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P6" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P6" s="30" t="inlineStr">
+        <is>
+          <t>Calculated from the index; reconciles with BCRD published monthly variation on 5,550/5,550 comparable values (all series).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="30" t="inlineStr">
@@ -1047,7 +1055,7 @@
       </c>
       <c r="K7" s="30" t="inlineStr">
         <is>
-          <t>BCRD (to validate)</t>
+          <t>BCRD — IPC base Oct 2019–Sep 2020 workbooks (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L7" s="30" t="inlineStr">
@@ -1067,10 +1075,14 @@
       </c>
       <c r="O7" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P7" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P7" s="30" t="inlineStr">
+        <is>
+          <t>Reconciles with BCRD published 12-month variation (headline and core, 808/808). NULL until 12 months of history (D4 rule).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="30" t="inlineStr">
@@ -1125,7 +1137,7 @@
       </c>
       <c r="K8" s="30" t="inlineStr">
         <is>
-          <t>BCRD (to validate)</t>
+          <t>BCRD — IPC base Oct 2019–Sep 2020 workbooks (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L8" s="30" t="inlineStr">
@@ -1145,10 +1157,14 @@
       </c>
       <c r="O8" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P8" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P8" s="30" t="inlineStr">
+        <is>
+          <t>Equals BCRD "con Dic." variation; reconciles 808/808. NULL in the first year of each series.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="30" t="inlineStr">
@@ -1178,7 +1194,7 @@
       </c>
       <c r="F9" s="30" t="inlineStr">
         <is>
-          <t>Use official published methodology/value; do not independently redefine</t>
+          <t>Same formulas applied to the official BCRD core CPI index</t>
         </is>
       </c>
       <c r="G9" s="30" t="inlineStr">
@@ -1203,7 +1219,7 @@
       </c>
       <c r="K9" s="30" t="inlineStr">
         <is>
-          <t>BCRD (to validate)</t>
+          <t>BCRD — IPC base Oct 2019–Sep 2020 workbooks (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L9" s="30" t="inlineStr">
@@ -1223,10 +1239,14 @@
       </c>
       <c r="O9" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P9" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P9" s="30" t="inlineStr">
+        <is>
+          <t>Official core index used as published (excludes volatile agricultural goods, alcohol, tobacco, fuels, administered and transport services); series_type = core.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
@@ -1256,7 +1276,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Period-over-period change using group CPI or official published rate</t>
+          <t>Same formulas applied to each expenditure-group index</t>
         </is>
       </c>
       <c r="G10" s="30" t="inlineStr">
@@ -1281,7 +1301,7 @@
       </c>
       <c r="K10" s="30" t="inlineStr">
         <is>
-          <t>BCRD (to validate)</t>
+          <t>BCRD — IPC base Oct 2019–Sep 2020 workbooks (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L10" s="30" t="inlineStr">
@@ -1301,10 +1321,14 @@
       </c>
       <c r="O10" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P10" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P10" s="30" t="inlineStr">
+        <is>
+          <t>12 COICOP-style groups as published by BCRD; series_type = expenditure_group. Regional CPI (4 regions) also available as series_type = region.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="30" t="inlineStr">
@@ -6189,6 +6213,252 @@
       <c r="P71" s="30" t="inlineStr">
         <is>
           <t>Do not use unauthorized scraping; source feasibility must be established first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="30" t="inlineStr">
+        <is>
+          <t>COL-001</t>
+        </is>
+      </c>
+      <c r="B72" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>How is the overall cost-of-living environment changing?</t>
+        </is>
+      </c>
+      <c r="D72" s="30" t="inlineStr">
+        <is>
+          <t>Family Basket Cost</t>
+        </is>
+      </c>
+      <c r="E72" s="30" t="inlineStr">
+        <is>
+          <t>Monthly cost in DOP of the BCRD family basket for the national household, each income quintile and each region.</t>
+        </is>
+      </c>
+      <c r="F72" s="30" t="inlineStr">
+        <is>
+          <t>Published BCRD value</t>
+        </is>
+      </c>
+      <c r="G72" s="30" t="inlineStr">
+        <is>
+          <t>DOP/month</t>
+        </is>
+      </c>
+      <c r="H72" s="30" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I72" s="30" t="inlineStr">
+        <is>
+          <t>Date; Segment type; Segment (quintile, national, region)</t>
+        </is>
+      </c>
+      <c r="J72" s="30" t="inlineStr">
+        <is>
+          <t>Basket cost by segment</t>
+        </is>
+      </c>
+      <c r="K72" s="30" t="inlineStr">
+        <is>
+          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="L72" s="30" t="inlineStr">
+        <is>
+          <t>gold.cost_of_living_metrics</t>
+        </is>
+      </c>
+      <c r="M72" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="N72" s="30" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="O72" s="30" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P72" s="30" t="inlineStr">
+        <is>
+          <t>ENGIH-2018 basket indexed by CPI. Quintile/national values before Oct-2020 are a BCRD retropolation (flagged).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="30" t="inlineStr">
+        <is>
+          <t>COL-002</t>
+        </is>
+      </c>
+      <c r="B73" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>How is the overall cost-of-living environment changing?</t>
+        </is>
+      </c>
+      <c r="D73" s="30" t="inlineStr">
+        <is>
+          <t>Basket Cost YoY %</t>
+        </is>
+      </c>
+      <c r="E73" s="30" t="inlineStr">
+        <is>
+          <t>Change in basket cost versus the same month one year earlier.</t>
+        </is>
+      </c>
+      <c r="F73" s="30" t="inlineStr">
+        <is>
+          <t>(Cost_t / Cost_t-12 - 1) * 100</t>
+        </is>
+      </c>
+      <c r="G73" s="30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H73" s="30" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I73" s="30" t="inlineStr">
+        <is>
+          <t>Date; Segment type; Segment</t>
+        </is>
+      </c>
+      <c r="J73" s="30" t="inlineStr">
+        <is>
+          <t>Basket cost history</t>
+        </is>
+      </c>
+      <c r="K73" s="30" t="inlineStr">
+        <is>
+          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="L73" s="30" t="inlineStr">
+        <is>
+          <t>gold.cost_of_living_metrics</t>
+        </is>
+      </c>
+      <c r="M73" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="N73" s="30" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="O73" s="30" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P73" s="30" t="inlineStr">
+        <is>
+          <t>National and regional values equal headline/regional CPI inflation (basket is CPI-indexed); the added value is the DOP level and the income-quintile view. Flag uses_retropolated_value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="30" t="inlineStr">
+        <is>
+          <t>COL-003</t>
+        </is>
+      </c>
+      <c r="B74" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>How is the overall cost-of-living environment changing?</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="inlineStr">
+        <is>
+          <t>Quintile 5 vs Quintile 1 Gap</t>
+        </is>
+      </c>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>Difference and ratio between the basket cost of the richest (Q5) and poorest (Q1) income quintile in the same month.</t>
+        </is>
+      </c>
+      <c r="F74" s="30" t="inlineStr">
+        <is>
+          <t>Q5 - Q1 (DOP); Q5 / Q1 (ratio)</t>
+        </is>
+      </c>
+      <c r="G74" s="30" t="inlineStr">
+        <is>
+          <t>DOP; ratio</t>
+        </is>
+      </c>
+      <c r="H74" s="30" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I74" s="30" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="J74" s="30" t="inlineStr">
+        <is>
+          <t>Basket cost Q1 and Q5</t>
+        </is>
+      </c>
+      <c r="K74" s="30" t="inlineStr">
+        <is>
+          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="L74" s="30" t="inlineStr">
+        <is>
+          <t>gold.cost_of_living_metrics</t>
+        </is>
+      </c>
+      <c r="M74" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="N74" s="30" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="O74" s="30" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P74" s="30" t="inlineStr">
+        <is>
+          <t>Month-level metric stored on the national row. Shows how household cost structure differs by income level.</t>
         </is>
       </c>
     </row>
@@ -6313,7 +6583,7 @@
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>
@@ -6340,7 +6610,7 @@
       </c>
       <c r="E6" s="28" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>
@@ -6367,7 +6637,7 @@
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>
@@ -6632,12 +6902,12 @@
       </c>
       <c r="D17" s="28" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="E17" s="28" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>
@@ -6667,7 +6937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7059,6 +7329,38 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>Housing &amp; Cost of Living</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(KPI_Catalog!$B$5:$B$200,A15)</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>COUNTIFS(KPI_Catalog!$B$5:$B$200,A15,KPI_Catalog!$N$5:$N$200,"MVP")</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>COUNTIFS(KPI_Catalog!$B$5:$B$200,A15,KPI_Catalog!$N$5:$N$200,"Phase 2")</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>COUNTIFS(KPI_Catalog!$B$5:$B$200,A15,KPI_Catalog!$O$5:$O$200,"Proposed")</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>COUNTIFS(KPI_Catalog!$B$5:$B$200,A15,KPI_Catalog!$O$5:$O$200,"Pending Source Validation")</f>
+        <v/>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add MICM fuel and Pro Consumidor pipelines, KPIs and Job tasks
</commit_message>
<xml_diff>
--- a/docs/03_Business_Questions_KPI_Catalog.xlsx
+++ b/docs/03_Business_Questions_KPI_Catalog.xlsx
@@ -2495,7 +2495,7 @@
       </c>
       <c r="G25" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H25" s="30" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="I25" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J25" s="30" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="K25" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L25" s="30" t="inlineStr">
@@ -2535,10 +2535,14 @@
       </c>
       <c r="O25" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P25" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P25" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="30" t="inlineStr">
@@ -2573,7 +2577,7 @@
       </c>
       <c r="G26" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H26" s="30" t="inlineStr">
@@ -2583,7 +2587,7 @@
       </c>
       <c r="I26" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J26" s="30" t="inlineStr">
@@ -2593,7 +2597,7 @@
       </c>
       <c r="K26" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L26" s="30" t="inlineStr">
@@ -2613,10 +2617,14 @@
       </c>
       <c r="O26" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P26" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P26" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="30" t="inlineStr">
@@ -2651,7 +2659,7 @@
       </c>
       <c r="G27" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H27" s="30" t="inlineStr">
@@ -2661,7 +2669,7 @@
       </c>
       <c r="I27" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J27" s="30" t="inlineStr">
@@ -2671,7 +2679,7 @@
       </c>
       <c r="K27" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L27" s="30" t="inlineStr">
@@ -2691,10 +2699,14 @@
       </c>
       <c r="O27" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P27" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P27" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="30" t="inlineStr">
@@ -2739,7 +2751,7 @@
       </c>
       <c r="I28" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J28" s="30" t="inlineStr">
@@ -2749,7 +2761,7 @@
       </c>
       <c r="K28" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L28" s="30" t="inlineStr">
@@ -2769,10 +2781,14 @@
       </c>
       <c r="O28" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P28" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P28" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="30" t="inlineStr">
@@ -2817,7 +2833,7 @@
       </c>
       <c r="I29" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J29" s="30" t="inlineStr">
@@ -2827,7 +2843,7 @@
       </c>
       <c r="K29" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L29" s="30" t="inlineStr">
@@ -2847,10 +2863,14 @@
       </c>
       <c r="O29" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P29" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P29" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. vs last published week of the previous month.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="30" t="inlineStr">
@@ -2895,7 +2915,7 @@
       </c>
       <c r="I30" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J30" s="30" t="inlineStr">
@@ -2905,7 +2925,7 @@
       </c>
       <c r="K30" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L30" s="30" t="inlineStr">
@@ -2925,10 +2945,14 @@
       </c>
       <c r="O30" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P30" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P30" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. vs the latest week starting 364–371 days earlier; NULL otherwise.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="30" t="inlineStr">
@@ -2973,7 +2997,7 @@
       </c>
       <c r="I31" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J31" s="30" t="inlineStr">
@@ -2983,7 +3007,7 @@
       </c>
       <c r="K31" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L31" s="30" t="inlineStr">
@@ -3003,10 +3027,14 @@
       </c>
       <c r="O31" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P31" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P31" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. vs last published week of the previous year.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="30" t="inlineStr">
@@ -3041,7 +3069,7 @@
       </c>
       <c r="G32" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H32" s="30" t="inlineStr">
@@ -3051,7 +3079,7 @@
       </c>
       <c r="I32" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J32" s="30" t="inlineStr">
@@ -3061,7 +3089,7 @@
       </c>
       <c r="K32" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L32" s="30" t="inlineStr">
@@ -3081,10 +3109,14 @@
       </c>
       <c r="O32" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P32" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P32" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. NULL until 4 weeks of history (D4).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="30" t="inlineStr">
@@ -3119,7 +3151,7 @@
       </c>
       <c r="G33" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H33" s="30" t="inlineStr">
@@ -3129,7 +3161,7 @@
       </c>
       <c r="I33" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J33" s="30" t="inlineStr">
@@ -3139,7 +3171,7 @@
       </c>
       <c r="K33" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L33" s="30" t="inlineStr">
@@ -3159,10 +3191,14 @@
       </c>
       <c r="O33" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P33" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P33" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. NULL until 12 weeks of history (D4).</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="30" t="inlineStr">
@@ -3197,7 +3233,7 @@
       </c>
       <c r="G34" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H34" s="30" t="inlineStr">
@@ -3207,7 +3243,7 @@
       </c>
       <c r="I34" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J34" s="30" t="inlineStr">
@@ -3217,7 +3253,7 @@
       </c>
       <c r="K34" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L34" s="30" t="inlineStr">
@@ -3237,10 +3273,14 @@
       </c>
       <c r="O34" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P34" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P34" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. Trailing 364 days; NULL with is_full_window_52w = false until a full year.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
@@ -3275,7 +3315,7 @@
       </c>
       <c r="G35" s="30" t="inlineStr">
         <is>
-          <t>DOP / unit</t>
+          <t>DOP/gallon</t>
         </is>
       </c>
       <c r="H35" s="30" t="inlineStr">
@@ -3285,7 +3325,7 @@
       </c>
       <c r="I35" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J35" s="30" t="inlineStr">
@@ -3295,7 +3335,7 @@
       </c>
       <c r="K35" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L35" s="30" t="inlineStr">
@@ -3315,10 +3355,14 @@
       </c>
       <c r="O35" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P35" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P35" s="30" t="inlineStr">
+        <is>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. Trailing 364 days; NULL with is_full_window_52w = false until a full year.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="30" t="inlineStr">
@@ -3363,7 +3407,7 @@
       </c>
       <c r="I36" s="30" t="inlineStr">
         <is>
-          <t>Date; Fuel Type; Unit</t>
+          <t>Price week; Fuel type</t>
         </is>
       </c>
       <c r="J36" s="30" t="inlineStr">
@@ -3373,7 +3417,7 @@
       </c>
       <c r="K36" s="30" t="inlineStr">
         <is>
-          <t>MICM (to validate)</t>
+          <t>MICM — precios-de-combustibles-2010-2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L36" s="30" t="inlineStr">
@@ -3393,12 +3437,12 @@
       </c>
       <c r="O36" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P36" s="30" t="inlineStr">
         <is>
-          <t>Volatility window/method to be finalized.</t>
+          <t>XLSX authoritative (CSV = XLSX rounded to whole pesos). Zero = not published. Std. dev. of weekly % changes over the trailing 12 weeks.</t>
         </is>
       </c>
     </row>
@@ -4392,12 +4436,12 @@
       </c>
       <c r="H49" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I49" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J49" s="30" t="inlineStr">
@@ -4407,7 +4451,7 @@
       </c>
       <c r="K49" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L49" s="30" t="inlineStr">
@@ -4427,10 +4471,14 @@
       </c>
       <c r="O49" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P49" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P49" s="30" t="inlineStr">
+        <is>
+          <t>Across retail segments, per month × product × presentation. 30 rows with years outside the report period rejected.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="30" t="inlineStr">
@@ -4470,12 +4518,12 @@
       </c>
       <c r="H50" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I50" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J50" s="30" t="inlineStr">
@@ -4485,7 +4533,7 @@
       </c>
       <c r="K50" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L50" s="30" t="inlineStr">
@@ -4505,10 +4553,14 @@
       </c>
       <c r="O50" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P50" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P50" s="30" t="inlineStr">
+        <is>
+          <t>Across retail segments.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="30" t="inlineStr">
@@ -4548,12 +4600,12 @@
       </c>
       <c r="H51" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I51" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J51" s="30" t="inlineStr">
@@ -4563,7 +4615,7 @@
       </c>
       <c r="K51" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L51" s="30" t="inlineStr">
@@ -4583,10 +4635,14 @@
       </c>
       <c r="O51" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P51" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P51" s="30" t="inlineStr">
+        <is>
+          <t>With cheapest_segment.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="30" t="inlineStr">
@@ -4626,12 +4682,12 @@
       </c>
       <c r="H52" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I52" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J52" s="30" t="inlineStr">
@@ -4641,7 +4697,7 @@
       </c>
       <c r="K52" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L52" s="30" t="inlineStr">
@@ -4661,10 +4717,14 @@
       </c>
       <c r="O52" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P52" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P52" s="30" t="inlineStr">
+        <is>
+          <t>With most_expensive_segment.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="30" t="inlineStr">
@@ -4704,12 +4764,12 @@
       </c>
       <c r="H53" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I53" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J53" s="30" t="inlineStr">
@@ -4719,7 +4779,7 @@
       </c>
       <c r="K53" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L53" s="30" t="inlineStr">
@@ -4739,12 +4799,12 @@
       </c>
       <c r="O53" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P53" s="30" t="inlineStr">
         <is>
-          <t>Comparability rules required across brand, presentation and unit.</t>
+          <t>Like-for-like: average of per-segment change for segments priced in both consecutive months (segment mix varies). NULL when none match.</t>
         </is>
       </c>
     </row>
@@ -4786,12 +4846,12 @@
       </c>
       <c r="H54" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I54" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J54" s="30" t="inlineStr">
@@ -4801,7 +4861,7 @@
       </c>
       <c r="K54" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L54" s="30" t="inlineStr">
@@ -4821,12 +4881,12 @@
       </c>
       <c r="O54" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Not Calculable</t>
         </is>
       </c>
       <c r="P54" s="30" t="inlineStr">
         <is>
-          <t>Comparability rules required across brand, presentation and unit.</t>
+          <t>Source covers 3 months (Jul–Sep 2026).</t>
         </is>
       </c>
     </row>
@@ -4868,12 +4928,12 @@
       </c>
       <c r="H55" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I55" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J55" s="30" t="inlineStr">
@@ -4883,7 +4943,7 @@
       </c>
       <c r="K55" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L55" s="30" t="inlineStr">
@@ -4903,12 +4963,12 @@
       </c>
       <c r="O55" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Not Calculable</t>
         </is>
       </c>
       <c r="P55" s="30" t="inlineStr">
         <is>
-          <t>Comparability rules required across brand, presentation and unit.</t>
+          <t>Source covers 3 months (Jul–Sep 2026).</t>
         </is>
       </c>
     </row>
@@ -4950,12 +5010,12 @@
       </c>
       <c r="H56" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I56" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J56" s="30" t="inlineStr">
@@ -4965,7 +5025,7 @@
       </c>
       <c r="K56" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L56" s="30" t="inlineStr">
@@ -4985,10 +5045,14 @@
       </c>
       <c r="O56" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P56" s="30" t="str"/>
+          <t>Not Calculable</t>
+        </is>
+      </c>
+      <c r="P56" s="30" t="inlineStr">
+        <is>
+          <t>Too few observations per product.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="30" t="inlineStr">
@@ -5028,12 +5092,12 @@
       </c>
       <c r="H57" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I57" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J57" s="30" t="inlineStr">
@@ -5043,7 +5107,7 @@
       </c>
       <c r="K57" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L57" s="30" t="inlineStr">
@@ -5063,12 +5127,12 @@
       </c>
       <c r="O57" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Not Calculable</t>
         </is>
       </c>
       <c r="P57" s="30" t="inlineStr">
         <is>
-          <t>Comparability rules required across brand, presentation and unit.</t>
+          <t>Source has no geography; price_spread_pct across retail segments provided instead (not regional).</t>
         </is>
       </c>
     </row>
@@ -5110,12 +5174,12 @@
       </c>
       <c r="H58" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I58" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Category; Brand; Presentation; Unit; Store; Municipality; Province; Region</t>
+          <t>Month; Product; Presentation; Retail segment</t>
         </is>
       </c>
       <c r="J58" s="30" t="inlineStr">
@@ -5125,7 +5189,7 @@
       </c>
       <c r="K58" s="30" t="inlineStr">
         <is>
-          <t>ProConsumidor / other official source (to validate)</t>
+          <t>Pro Consumidor — Precios Productos de Primera Necesidad, Jul–Sep 2026 XLSX (validated 2026-10-23)</t>
         </is>
       </c>
       <c r="L58" s="30" t="inlineStr">
@@ -5150,7 +5214,7 @@
       </c>
       <c r="P58" s="30" t="inlineStr">
         <is>
-          <t>Comparability rules required across brand, presentation and unit.</t>
+          <t>Needs category mapping and weighting methodology.</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6755,7 @@
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6836,7 @@
       </c>
       <c r="E12" s="28" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Partially Validated</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add MEM electricity pipeline (ENE-001..009), Job tasks and Power BI page
</commit_message>
<xml_diff>
--- a/docs/03_Business_Questions_KPI_Catalog.xlsx
+++ b/docs/03_Business_Questions_KPI_Catalog.xlsx
@@ -691,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P74"/>
+  <dimension ref="A1:P78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5806,47 +5806,47 @@
       </c>
       <c r="D66" s="30" t="inlineStr">
         <is>
-          <t>Electricity Tariff</t>
+          <t>Electricity Tariff (applied)</t>
         </is>
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Published tariff applicable to the selected customer/tariff category.</t>
+          <t>Regulated tariff charged to the customer, by tariff, concept and distributor.</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Published tariff</t>
+          <t>Applied tariff from SIE resolutions (MEM annex)</t>
         </is>
       </c>
       <c r="G66" s="30" t="inlineStr">
         <is>
-          <t>DOP/kWh or source unit</t>
+          <t>RD$ per unit of the concept</t>
         </is>
       </c>
       <c r="H66" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly (quarterly resolutions)</t>
         </is>
       </c>
       <c r="I66" s="30" t="inlineStr">
         <is>
-          <t>Date; Tariff Category; Distributor/Region (if available)</t>
+          <t>Month; Distributor; Tariff; Concept</t>
         </is>
       </c>
       <c r="J66" s="30" t="inlineStr">
         <is>
-          <t>Tariff; category; date; unit</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K66" s="30" t="inlineStr">
         <is>
-          <t>SIE / EDEs / official source (to validate)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L66" s="30" t="inlineStr">
         <is>
-          <t>gold.energy_price_metrics</t>
+          <t>gold.electricity_tariff_monthly</t>
         </is>
       </c>
       <c r="M66" s="30" t="inlineStr">
@@ -5861,12 +5861,12 @@
       </c>
       <c r="O66" s="30" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P66" s="30" t="inlineStr">
         <is>
-          <t>Scope depends on historical source availability and tariff comparability.</t>
+          <t>Before Oct 2021 one applied value for all distributors.</t>
         </is>
       </c>
     </row>
@@ -5888,17 +5888,17 @@
       </c>
       <c r="D67" s="30" t="inlineStr">
         <is>
-          <t>MoM Tariff Change %</t>
+          <t>Reference vs Applied Tariff Gap %</t>
         </is>
       </c>
       <c r="E67" s="30" t="inlineStr">
         <is>
-          <t>Monthly percentage change in comparable tariff.</t>
+          <t>Difference between the cost-based reference tariff and the applied tariff.</t>
         </is>
       </c>
       <c r="F67" s="30" t="inlineStr">
         <is>
-          <t>(Tariff_t / Tariff_prev_month - 1) * 100</t>
+          <t>(Reference / Applied - 1) * 100</t>
         </is>
       </c>
       <c r="G67" s="30" t="inlineStr">
@@ -5908,27 +5908,27 @@
       </c>
       <c r="H67" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I67" s="30" t="inlineStr">
         <is>
-          <t>Date; Tariff Category; Distributor/Region (if available)</t>
+          <t>Month; Distributor; Tariff; Concept</t>
         </is>
       </c>
       <c r="J67" s="30" t="inlineStr">
         <is>
-          <t>Tariff; category; date; unit</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K67" s="30" t="inlineStr">
         <is>
-          <t>SIE / EDEs / official source (to validate)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L67" s="30" t="inlineStr">
         <is>
-          <t>gold.energy_price_metrics</t>
+          <t>gold.electricity_tariff_monthly</t>
         </is>
       </c>
       <c r="M67" s="30" t="inlineStr">
@@ -5943,12 +5943,12 @@
       </c>
       <c r="O67" s="30" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P67" s="30" t="inlineStr">
         <is>
-          <t>Scope depends on historical source availability and tariff comparability.</t>
+          <t>Proxy of the tariff subsidy; reference = 'tarifa indexada' before Oct 2021.</t>
         </is>
       </c>
     </row>
@@ -5970,47 +5970,47 @@
       </c>
       <c r="D68" s="30" t="inlineStr">
         <is>
-          <t>YoY Tariff Change %</t>
+          <t>Typical Residential Bill (BTS-1)</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Year-over-year percentage change in comparable tariff.</t>
+          <t>Monthly bill for a BTS-1 customer consuming 200 or 300 kWh.</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>(Tariff_t / Tariff_t-1year - 1) * 100</t>
+          <t>Fixed charge (101+ kWh) + 200 * block 1 (+ 100 * block 2)</t>
         </is>
       </c>
       <c r="G68" s="30" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>RD$/month</t>
         </is>
       </c>
       <c r="H68" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I68" s="30" t="inlineStr">
         <is>
-          <t>Date; Tariff Category; Distributor/Region (if available)</t>
+          <t>Month; Distributor; Monthly kWh</t>
         </is>
       </c>
       <c r="J68" s="30" t="inlineStr">
         <is>
-          <t>Tariff; category; date; unit</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K68" s="30" t="inlineStr">
         <is>
-          <t>SIE / EDEs / official source (to validate)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L68" s="30" t="inlineStr">
         <is>
-          <t>gold.energy_price_metrics</t>
+          <t>gold.electricity_bts1_bill</t>
         </is>
       </c>
       <c r="M68" s="30" t="inlineStr">
@@ -6025,12 +6025,12 @@
       </c>
       <c r="O68" s="30" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P68" s="30" t="inlineStr">
         <is>
-          <t>Scope depends on historical source availability and tariff comparability.</t>
+          <t>Applied and reference tariff; excludes taxes and other charges.</t>
         </is>
       </c>
     </row>
@@ -6052,17 +6052,17 @@
       </c>
       <c r="D69" s="30" t="inlineStr">
         <is>
-          <t>YTD Tariff Change %</t>
+          <t>Typical Bill YoY %</t>
         </is>
       </c>
       <c r="E69" s="30" t="inlineStr">
         <is>
-          <t>Percentage change versus prior-year-end tariff.</t>
+          <t>Year-over-year change of the typical BTS-1 bill.</t>
         </is>
       </c>
       <c r="F69" s="30" t="inlineStr">
         <is>
-          <t>(Tariff_t / Tariff_last_prev_year - 1) * 100</t>
+          <t>(Bill_t / Bill_t-12 - 1) * 100</t>
         </is>
       </c>
       <c r="G69" s="30" t="inlineStr">
@@ -6072,27 +6072,27 @@
       </c>
       <c r="H69" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I69" s="30" t="inlineStr">
         <is>
-          <t>Date; Tariff Category; Distributor/Region (if available)</t>
+          <t>Month; Distributor; Monthly kWh</t>
         </is>
       </c>
       <c r="J69" s="30" t="inlineStr">
         <is>
-          <t>Tariff; category; date; unit</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K69" s="30" t="inlineStr">
         <is>
-          <t>SIE / EDEs / official source (to validate)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L69" s="30" t="inlineStr">
         <is>
-          <t>gold.energy_price_metrics</t>
+          <t>gold.electricity_bts1_bill</t>
         </is>
       </c>
       <c r="M69" s="30" t="inlineStr">
@@ -6107,14 +6107,10 @@
       </c>
       <c r="O69" s="30" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
-        </is>
-      </c>
-      <c r="P69" s="30" t="inlineStr">
-        <is>
-          <t>Scope depends on historical source availability and tariff comparability.</t>
-        </is>
-      </c>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P69" s="30" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="30" t="inlineStr">
@@ -6134,17 +6130,17 @@
       </c>
       <c r="D70" s="30" t="inlineStr">
         <is>
-          <t>Average Cost per kWh</t>
+          <t>Average Cost per kWh (selling price)</t>
         </is>
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Average comparable electricity cost per kWh for selected category.</t>
+          <t>Average selling price of the state distributors per kWh billed.</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>AVG(cost_per_kWh) where concept is comparable</t>
+          <t>Published MEM average selling price</t>
         </is>
       </c>
       <c r="G70" s="30" t="inlineStr">
@@ -6154,27 +6150,27 @@
       </c>
       <c r="H70" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I70" s="30" t="inlineStr">
         <is>
-          <t>Date; Tariff Category; Distributor/Region (if available)</t>
+          <t>Month; Distributor</t>
         </is>
       </c>
       <c r="J70" s="30" t="inlineStr">
         <is>
-          <t>Tariff; category; date; unit</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K70" s="30" t="inlineStr">
         <is>
-          <t>SIE / EDEs / official source (to validate)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L70" s="30" t="inlineStr">
         <is>
-          <t>gold.energy_price_metrics</t>
+          <t>gold.electricity_metrics</t>
         </is>
       </c>
       <c r="M70" s="30" t="inlineStr">
@@ -6189,79 +6185,79 @@
       </c>
       <c r="O70" s="30" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P70" s="30" t="inlineStr">
         <is>
-          <t>Scope depends on historical source availability and tariff comparability.</t>
+          <t>Reconciles with MEM PDF May 2026 (Edenorte 10.13, Edesur 10.51).</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="30" t="inlineStr">
         <is>
-          <t>HOU-001</t>
+          <t>ENE-006</t>
         </is>
       </c>
       <c r="B71" s="30" t="inlineStr">
         <is>
-          <t>Housing / Rentals</t>
+          <t>Energy / Electricity</t>
         </is>
       </c>
       <c r="C71" s="30" t="inlineStr">
         <is>
-          <t>How are rental prices and housing costs evolving?</t>
+          <t>How are electricity and energy costs evolving?</t>
         </is>
       </c>
       <c r="D71" s="30" t="inlineStr">
         <is>
-          <t>Median Rental Asking Price</t>
+          <t>Average Selling Price MoM % / YoY %</t>
         </is>
       </c>
       <c r="E71" s="30" t="inlineStr">
         <is>
-          <t>Median observed asking rent for comparable properties within a geography/property segment.</t>
+          <t>Change of the average selling price per kWh.</t>
         </is>
       </c>
       <c r="F71" s="30" t="inlineStr">
         <is>
-          <t>MEDIAN(asking_rent)</t>
+          <t>(P_t / P_t-1 - 1) * 100; (P_t / P_t-12 - 1) * 100</t>
         </is>
       </c>
       <c r="G71" s="30" t="inlineStr">
         <is>
-          <t>DOP/month</t>
+          <t>%</t>
         </is>
       </c>
       <c r="H71" s="30" t="inlineStr">
         <is>
-          <t>Monthly / Source-dependent</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="I71" s="30" t="inlineStr">
         <is>
-          <t>Date; Property Type; Bedrooms; Municipality; Sector</t>
+          <t>Month; Distributor</t>
         </is>
       </c>
       <c r="J71" s="30" t="inlineStr">
         <is>
-          <t>Asking rent; date; property attributes; location</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K71" s="30" t="inlineStr">
         <is>
-          <t>TBD — legally/technically appropriate source</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L71" s="30" t="inlineStr">
         <is>
-          <t>gold.housing_price_metrics</t>
+          <t>gold.electricity_metrics</t>
         </is>
       </c>
       <c r="M71" s="30" t="inlineStr">
         <is>
-          <t>Housing &amp; Cost of Living</t>
+          <t>Energy &amp; Electricity</t>
         </is>
       </c>
       <c r="N71" s="30" t="inlineStr">
@@ -6271,49 +6267,45 @@
       </c>
       <c r="O71" s="30" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
-        </is>
-      </c>
-      <c r="P71" s="30" t="inlineStr">
-        <is>
-          <t>Do not use unauthorized scraping; source feasibility must be established first.</t>
-        </is>
-      </c>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P71" s="30" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="30" t="inlineStr">
         <is>
-          <t>COL-001</t>
+          <t>ENE-007</t>
         </is>
       </c>
       <c r="B72" s="30" t="inlineStr">
         <is>
-          <t>Cost of Living</t>
+          <t>Energy / Electricity</t>
         </is>
       </c>
       <c r="C72" s="30" t="inlineStr">
         <is>
-          <t>How is the overall cost-of-living environment changing?</t>
+          <t>How are electricity and energy costs evolving?</t>
         </is>
       </c>
       <c r="D72" s="30" t="inlineStr">
         <is>
-          <t>Family Basket Cost</t>
+          <t>Average Purchase Price and Margin</t>
         </is>
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Monthly cost in DOP of the BCRD family basket for the national household, each income quintile and each region.</t>
+          <t>Average price paid by the distributors for energy, and the selling minus purchase margin.</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Published BCRD value</t>
+          <t>Published purchase price; sell - buy</t>
         </is>
       </c>
       <c r="G72" s="30" t="inlineStr">
         <is>
-          <t>DOP/month</t>
+          <t>US¢/kWh</t>
         </is>
       </c>
       <c r="H72" s="30" t="inlineStr">
@@ -6323,32 +6315,32 @@
       </c>
       <c r="I72" s="30" t="inlineStr">
         <is>
-          <t>Date; Segment type; Segment (quintile, national, region)</t>
+          <t>Month; Distributor</t>
         </is>
       </c>
       <c r="J72" s="30" t="inlineStr">
         <is>
-          <t>Basket cost by segment</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K72" s="30" t="inlineStr">
         <is>
-          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L72" s="30" t="inlineStr">
         <is>
-          <t>gold.cost_of_living_metrics</t>
+          <t>gold.electricity_metrics</t>
         </is>
       </c>
       <c r="M72" s="30" t="inlineStr">
         <is>
-          <t>Cost of Living</t>
+          <t>Energy &amp; Electricity</t>
         </is>
       </c>
       <c r="N72" s="30" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="O72" s="30" t="inlineStr">
@@ -6356,41 +6348,37 @@
           <t>Validated</t>
         </is>
       </c>
-      <c r="P72" s="30" t="inlineStr">
-        <is>
-          <t>ENGIH-2018 basket indexed by CPI. Quintile/national values before Oct-2020 are a BCRD retropolation (flagged).</t>
-        </is>
-      </c>
+      <c r="P72" s="30" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="30" t="inlineStr">
         <is>
-          <t>COL-002</t>
+          <t>ENE-008</t>
         </is>
       </c>
       <c r="B73" s="30" t="inlineStr">
         <is>
-          <t>Cost of Living</t>
+          <t>Energy / Electricity</t>
         </is>
       </c>
       <c r="C73" s="30" t="inlineStr">
         <is>
-          <t>How is the overall cost-of-living environment changing?</t>
+          <t>How are electricity and energy costs evolving?</t>
         </is>
       </c>
       <c r="D73" s="30" t="inlineStr">
         <is>
-          <t>Basket Cost YoY %</t>
+          <t>Energy Losses %</t>
         </is>
       </c>
       <c r="E73" s="30" t="inlineStr">
         <is>
-          <t>Change in basket cost versus the same month one year earlier.</t>
+          <t>Share of energy bought that is not billed.</t>
         </is>
       </c>
       <c r="F73" s="30" t="inlineStr">
         <is>
-          <t>(Cost_t / Cost_t-12 - 1) * 100</t>
+          <t>Published losses % (month and 12-month rolling)</t>
         </is>
       </c>
       <c r="G73" s="30" t="inlineStr">
@@ -6405,32 +6393,32 @@
       </c>
       <c r="I73" s="30" t="inlineStr">
         <is>
-          <t>Date; Segment type; Segment</t>
+          <t>Month; Distributor</t>
         </is>
       </c>
       <c r="J73" s="30" t="inlineStr">
         <is>
-          <t>Basket cost history</t>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
         </is>
       </c>
       <c r="K73" s="30" t="inlineStr">
         <is>
-          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L73" s="30" t="inlineStr">
         <is>
-          <t>gold.cost_of_living_metrics</t>
+          <t>gold.electricity_metrics</t>
         </is>
       </c>
       <c r="M73" s="30" t="inlineStr">
         <is>
-          <t>Cost of Living</t>
+          <t>Energy &amp; Electricity</t>
         </is>
       </c>
       <c r="N73" s="30" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="O73" s="30" t="inlineStr">
@@ -6438,89 +6426,409 @@
           <t>Validated</t>
         </is>
       </c>
-      <c r="P73" s="30" t="inlineStr">
-        <is>
-          <t>National and regional values equal headline/regional CPI inflation (basket is CPI-indexed); the added value is the DOP level and the income-quintile view. Flag uses_retropolated_value.</t>
-        </is>
-      </c>
+      <c r="P73" s="30" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="30" t="inlineStr">
         <is>
+          <t>ENE-009</t>
+        </is>
+      </c>
+      <c r="B74" s="30" t="inlineStr">
+        <is>
+          <t>Energy / Electricity</t>
+        </is>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>How are electricity and energy costs evolving?</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="inlineStr">
+        <is>
+          <t>Collection % and CRI %</t>
+        </is>
+      </c>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>Collection rate and cash recovery index, 12-month rolling.</t>
+        </is>
+      </c>
+      <c r="F74" s="30" t="inlineStr">
+        <is>
+          <t>Published rolling indicators</t>
+        </is>
+      </c>
+      <c r="G74" s="30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H74" s="30" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I74" s="30" t="inlineStr">
+        <is>
+          <t>Month; Distributor</t>
+        </is>
+      </c>
+      <c r="J74" s="30" t="inlineStr">
+        <is>
+          <t>MEM annex sheets EDE's and Nuevo Regimen tarifario</t>
+        </is>
+      </c>
+      <c r="K74" s="30" t="inlineStr">
+        <is>
+          <t>MEM — Informe de Desempeño EEE, Anexos julio 2026 (validated 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L74" s="30" t="inlineStr">
+        <is>
+          <t>gold.electricity_metrics</t>
+        </is>
+      </c>
+      <c r="M74" s="30" t="inlineStr">
+        <is>
+          <t>Energy &amp; Electricity</t>
+        </is>
+      </c>
+      <c r="N74" s="30" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="O74" s="30" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P74" s="30" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="30" t="inlineStr">
+        <is>
+          <t>HOU-001</t>
+        </is>
+      </c>
+      <c r="B75" s="30" t="inlineStr">
+        <is>
+          <t>Housing / Rentals</t>
+        </is>
+      </c>
+      <c r="C75" s="30" t="inlineStr">
+        <is>
+          <t>How are rental prices and housing costs evolving?</t>
+        </is>
+      </c>
+      <c r="D75" s="30" t="inlineStr">
+        <is>
+          <t>Median Rental Asking Price</t>
+        </is>
+      </c>
+      <c r="E75" s="30" t="inlineStr">
+        <is>
+          <t>Median observed asking rent for comparable properties within a geography/property segment.</t>
+        </is>
+      </c>
+      <c r="F75" s="30" t="inlineStr">
+        <is>
+          <t>MEDIAN(asking_rent)</t>
+        </is>
+      </c>
+      <c r="G75" s="30" t="inlineStr">
+        <is>
+          <t>DOP/month</t>
+        </is>
+      </c>
+      <c r="H75" s="30" t="inlineStr">
+        <is>
+          <t>Monthly / Source-dependent</t>
+        </is>
+      </c>
+      <c r="I75" s="30" t="inlineStr">
+        <is>
+          <t>Date; Property Type; Bedrooms; Municipality; Sector</t>
+        </is>
+      </c>
+      <c r="J75" s="30" t="inlineStr">
+        <is>
+          <t>Asking rent; date; property attributes; location</t>
+        </is>
+      </c>
+      <c r="K75" s="30" t="inlineStr">
+        <is>
+          <t>TBD — legally/technically appropriate source</t>
+        </is>
+      </c>
+      <c r="L75" s="30" t="inlineStr">
+        <is>
+          <t>gold.housing_price_metrics</t>
+        </is>
+      </c>
+      <c r="M75" s="30" t="inlineStr">
+        <is>
+          <t>Housing &amp; Cost of Living</t>
+        </is>
+      </c>
+      <c r="N75" s="30" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="O75" s="30" t="inlineStr">
+        <is>
+          <t>Pending Source Validation</t>
+        </is>
+      </c>
+      <c r="P75" s="30" t="inlineStr">
+        <is>
+          <t>Do not use unauthorized scraping; source feasibility must be established first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>COL-001</t>
+        </is>
+      </c>
+      <c r="B76" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>How is the overall cost-of-living environment changing?</t>
+        </is>
+      </c>
+      <c r="D76" s="30" t="inlineStr">
+        <is>
+          <t>Family Basket Cost</t>
+        </is>
+      </c>
+      <c r="E76" s="30" t="inlineStr">
+        <is>
+          <t>Monthly cost in DOP of the BCRD family basket for the national household, each income quintile and each region.</t>
+        </is>
+      </c>
+      <c r="F76" s="30" t="inlineStr">
+        <is>
+          <t>Published BCRD value</t>
+        </is>
+      </c>
+      <c r="G76" s="30" t="inlineStr">
+        <is>
+          <t>DOP/month</t>
+        </is>
+      </c>
+      <c r="H76" s="30" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I76" s="30" t="inlineStr">
+        <is>
+          <t>Date; Segment type; Segment (quintile, national, region)</t>
+        </is>
+      </c>
+      <c r="J76" s="30" t="inlineStr">
+        <is>
+          <t>Basket cost by segment</t>
+        </is>
+      </c>
+      <c r="K76" s="30" t="inlineStr">
+        <is>
+          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="L76" s="30" t="inlineStr">
+        <is>
+          <t>gold.cost_of_living_metrics</t>
+        </is>
+      </c>
+      <c r="M76" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="N76" s="30" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="O76" s="30" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P76" s="30" t="inlineStr">
+        <is>
+          <t>ENGIH-2018 basket indexed by CPI. Quintile/national values before Oct-2020 are a BCRD retropolation (flagged).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>COL-002</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>How is the overall cost-of-living environment changing?</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>Basket Cost YoY %</t>
+        </is>
+      </c>
+      <c r="E77" s="30" t="inlineStr">
+        <is>
+          <t>Change in basket cost versus the same month one year earlier.</t>
+        </is>
+      </c>
+      <c r="F77" s="30" t="inlineStr">
+        <is>
+          <t>(Cost_t / Cost_t-12 - 1) * 100</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H77" s="30" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="I77" s="30" t="inlineStr">
+        <is>
+          <t>Date; Segment type; Segment</t>
+        </is>
+      </c>
+      <c r="J77" s="30" t="inlineStr">
+        <is>
+          <t>Basket cost history</t>
+        </is>
+      </c>
+      <c r="K77" s="30" t="inlineStr">
+        <is>
+          <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
+        </is>
+      </c>
+      <c r="L77" s="30" t="inlineStr">
+        <is>
+          <t>gold.cost_of_living_metrics</t>
+        </is>
+      </c>
+      <c r="M77" s="30" t="inlineStr">
+        <is>
+          <t>Cost of Living</t>
+        </is>
+      </c>
+      <c r="N77" s="30" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="O77" s="30" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P77" s="30" t="inlineStr">
+        <is>
+          <t>National and regional values equal headline/regional CPI inflation (basket is CPI-indexed); the added value is the DOP level and the income-quintile view. Flag uses_retropolated_value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
+        <is>
           <t>COL-003</t>
         </is>
       </c>
-      <c r="B74" s="30" t="inlineStr">
+      <c r="B78" s="30" t="inlineStr">
         <is>
           <t>Cost of Living</t>
         </is>
       </c>
-      <c r="C74" s="30" t="inlineStr">
+      <c r="C78" s="30" t="inlineStr">
         <is>
           <t>How is the overall cost-of-living environment changing?</t>
         </is>
       </c>
-      <c r="D74" s="30" t="inlineStr">
+      <c r="D78" s="30" t="inlineStr">
         <is>
           <t>Quintile 5 vs Quintile 1 Gap</t>
         </is>
       </c>
-      <c r="E74" s="30" t="inlineStr">
+      <c r="E78" s="30" t="inlineStr">
         <is>
           <t>Difference and ratio between the basket cost of the richest (Q5) and poorest (Q1) income quintile in the same month.</t>
         </is>
       </c>
-      <c r="F74" s="30" t="inlineStr">
+      <c r="F78" s="30" t="inlineStr">
         <is>
           <t>Q5 - Q1 (DOP); Q5 / Q1 (ratio)</t>
         </is>
       </c>
-      <c r="G74" s="30" t="inlineStr">
+      <c r="G78" s="30" t="inlineStr">
         <is>
           <t>DOP; ratio</t>
         </is>
       </c>
-      <c r="H74" s="30" t="inlineStr">
+      <c r="H78" s="30" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="I74" s="30" t="inlineStr">
+      <c r="I78" s="30" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="J74" s="30" t="inlineStr">
+      <c r="J78" s="30" t="inlineStr">
         <is>
           <t>Basket cost Q1 and Q5</t>
         </is>
       </c>
-      <c r="K74" s="30" t="inlineStr">
+      <c r="K78" s="30" t="inlineStr">
         <is>
           <t>BCRD — Costo de la Canasta Familiar (validated 2026-10-23)</t>
         </is>
       </c>
-      <c r="L74" s="30" t="inlineStr">
+      <c r="L78" s="30" t="inlineStr">
         <is>
           <t>gold.cost_of_living_metrics</t>
         </is>
       </c>
-      <c r="M74" s="30" t="inlineStr">
+      <c r="M78" s="30" t="inlineStr">
         <is>
           <t>Cost of Living</t>
         </is>
       </c>
-      <c r="N74" s="30" t="inlineStr">
+      <c r="N78" s="30" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="O74" s="30" t="inlineStr">
+      <c r="O78" s="30" t="inlineStr">
         <is>
           <t>Validated</t>
         </is>
       </c>
-      <c r="P74" s="30" t="inlineStr">
+      <c r="P78" s="30" t="inlineStr">
         <is>
           <t>Month-level metric stored on the national row. Shows how household cost structure differs by income level.</t>
         </is>
@@ -6890,7 +7198,7 @@
       </c>
       <c r="E14" s="28" t="inlineStr">
         <is>
-          <t>Pending Source Validation</t>
+          <t>Validated</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Ministry of Agriculture market prices pipeline (AGR-001..005, AGR-007)
- Automatic download from datos.gob.do (retail .xls, wholesale .xlsx and CSVs), Auto Loader Bronze
- Silver: market unpivot, controlled dictionaries for week/month/year typos, 10 product groups, not-quoted vs price, Excel vs CSV reconciliation
- Gold: monthly prices by channel/market/product/unit with MoM, YoY, YTD, volatility and market difference; product-group view
- Main Job: sixth chain (25 tasks); KPI catalog and docs updated
</commit_message>
<xml_diff>
--- a/docs/03_Business_Questions_KPI_Catalog.xlsx
+++ b/docs/03_Business_Questions_KPI_Catalog.xlsx
@@ -756,6 +756,7 @@
       <c r="O2" s="1" t="n"/>
       <c r="P2" s="1" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -5261,7 +5262,7 @@
       </c>
       <c r="I59" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J59" s="30" t="inlineStr">
@@ -5271,12 +5272,12 @@
       </c>
       <c r="K59" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L59" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly</t>
         </is>
       </c>
       <c r="M59" s="30" t="inlineStr">
@@ -5291,10 +5292,14 @@
       </c>
       <c r="O59" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="P59" s="30" t="str"/>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="P59" s="30" t="inlineStr">
+        <is>
+          <t>Monthly average of weekly quotes per market; 0 and N/D = not quoted.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="30" t="inlineStr">
@@ -5339,7 +5344,7 @@
       </c>
       <c r="I60" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J60" s="30" t="inlineStr">
@@ -5349,12 +5354,12 @@
       </c>
       <c r="K60" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L60" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly; gold.agri_rubro_monthly</t>
         </is>
       </c>
       <c r="M60" s="30" t="inlineStr">
@@ -5369,12 +5374,12 @@
       </c>
       <c r="O60" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P60" s="30" t="inlineStr">
         <is>
-          <t>Requires unit and market-level comparability validation.</t>
+          <t>Same channel, market, product and unit; previous month / year / December must exist.</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5426,7 @@
       </c>
       <c r="I61" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J61" s="30" t="inlineStr">
@@ -5431,12 +5436,12 @@
       </c>
       <c r="K61" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L61" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly; gold.agri_rubro_monthly</t>
         </is>
       </c>
       <c r="M61" s="30" t="inlineStr">
@@ -5451,12 +5456,12 @@
       </c>
       <c r="O61" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P61" s="30" t="inlineStr">
         <is>
-          <t>Requires unit and market-level comparability validation.</t>
+          <t>Same channel, market, product and unit; previous month / year / December must exist.</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5508,7 @@
       </c>
       <c r="I62" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J62" s="30" t="inlineStr">
@@ -5513,12 +5518,12 @@
       </c>
       <c r="K62" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L62" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly</t>
         </is>
       </c>
       <c r="M62" s="30" t="inlineStr">
@@ -5533,12 +5538,12 @@
       </c>
       <c r="O62" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P62" s="30" t="inlineStr">
         <is>
-          <t>Requires unit and market-level comparability validation.</t>
+          <t>Same channel, market, product and unit; previous month / year / December must exist.</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5590,7 @@
       </c>
       <c r="I63" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J63" s="30" t="inlineStr">
@@ -5595,12 +5600,12 @@
       </c>
       <c r="K63" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L63" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly</t>
         </is>
       </c>
       <c r="M63" s="30" t="inlineStr">
@@ -5615,12 +5620,12 @@
       </c>
       <c r="O63" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated</t>
         </is>
       </c>
       <c r="P63" s="30" t="inlineStr">
         <is>
-          <t>Requires unit and market-level comparability validation.</t>
+          <t>Std. dev. of MoM % over the last 12 months, min 6 values.</t>
         </is>
       </c>
     </row>
@@ -5667,7 +5672,7 @@
       </c>
       <c r="I64" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J64" s="30" t="inlineStr">
@@ -5677,12 +5682,12 @@
       </c>
       <c r="K64" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L64" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly</t>
         </is>
       </c>
       <c r="M64" s="30" t="inlineStr">
@@ -5702,7 +5707,7 @@
       </c>
       <c r="P64" s="30" t="inlineStr">
         <is>
-          <t>Requires unit and market-level comparability validation.</t>
+          <t>Not calculated: seasonal methodology not defined.</t>
         </is>
       </c>
     </row>
@@ -5724,7 +5729,7 @@
       </c>
       <c r="D65" s="30" t="inlineStr">
         <is>
-          <t>Regional Price Difference %</t>
+          <t>Market Price Difference %</t>
         </is>
       </c>
       <c r="E65" s="30" t="inlineStr">
@@ -5749,7 +5754,7 @@
       </c>
       <c r="I65" s="30" t="inlineStr">
         <is>
-          <t>Date; Product; Unit; Market; Municipality; Province; Region</t>
+          <t>Month; Channel (retail/wholesale); Market (7 Gran Santo Domingo markets); Product group (rubro); Product; Unit</t>
         </is>
       </c>
       <c r="J65" s="30" t="inlineStr">
@@ -5759,12 +5764,12 @@
       </c>
       <c r="K65" s="30" t="inlineStr">
         <is>
-          <t>Ministry of Agriculture / public data source (to validate)</t>
+          <t>Ministry of Agriculture — Informe Precios de Mercado Interdiario 2017-2026, datos.gob.do (validated 2026-10-24)</t>
         </is>
       </c>
       <c r="L65" s="30" t="inlineStr">
         <is>
-          <t>gold.agricultural_price_metrics</t>
+          <t>gold.agri_price_monthly</t>
         </is>
       </c>
       <c r="M65" s="30" t="inlineStr">
@@ -5779,12 +5784,12 @@
       </c>
       <c r="O65" s="30" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Validated (market level)</t>
         </is>
       </c>
       <c r="P65" s="30" t="inlineStr">
         <is>
-          <t>Requires unit and market-level comparability validation.</t>
+          <t>Source has markets of Gran Santo Domingo, not regions: (market price / average of retail markets - 1) * 100.</t>
         </is>
       </c>
     </row>

</xml_diff>